<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales_cobertura)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_cobertura/plot_comunal_cobertura_2018_biobio.xlsx
+++ b/output/graficos_regionales_cobertura/plot_comunal_cobertura_2018_biobio.xlsx
@@ -78,7 +78,7 @@
     <t xml:space="preserve">Chiguayante</t>
   </si>
   <si>
-    <t xml:space="preserve">Los Alamos</t>
+    <t xml:space="preserve">Los Álamos</t>
   </si>
   <si>
     <t xml:space="preserve">Mulchén</t>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">Tomé</t>
   </si>
   <si>
-    <t xml:space="preserve">Los Angeles</t>
+    <t xml:space="preserve">Los Ángeles</t>
   </si>
   <si>
     <t xml:space="preserve">Arauco</t>
@@ -138,7 +138,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-27 21:43</t>
+    <t xml:space="preserve">2026-10-05 05:40</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>

</xml_diff>